<commit_message>
docs: update quantum chemistry visualization survey
</commit_message>
<xml_diff>
--- a/pyscf_quantum_chemistry_visualization_research_2026-07-19.xlsx
+++ b/pyscf_quantum_chemistry_visualization_research_2026-07-19.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R8feca3b537184ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心文献" sheetId="2" r:id="R9801916fc02e4e77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件矩阵" sheetId="3" r:id="R1de69cc7e07c4fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷题库" sheetId="4" r:id="R7dd6864c6d714acc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验证矩阵" sheetId="5" r:id="R265cca4f40b84997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R0b9e11b89d1f4ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心文献" sheetId="2" r:id="Rbe4ae855ed8f443f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件矩阵" sheetId="3" r:id="R47bbef6c080c43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷题库" sheetId="4" r:id="R655fbeae2d1746fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验证矩阵" sheetId="5" r:id="Rd42fa0551dfb4bbc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,67 +127,27 @@
   <x:borders count="18">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="108">
+  <x:cellXfs count="109">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -452,6 +412,9 @@
     <x:xf numFmtId="200" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -463,7 +426,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -473,7 +436,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -483,7 +446,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -494,7 +457,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -504,7 +467,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -525,17 +488,14 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr/>
               <a:t>文献主题分布</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:varyColors val="0"/>
@@ -666,7 +626,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R212ac673ace94608"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5fcfb790519d47e3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -803,9 +763,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -985,13 +945,11 @@
         <x:v>PySCF已有高质量软件论文、活跃版本、广泛方法覆盖、周期体系和GPU/工业应用证据。它在方法开发、自动化和Python生态中的可信度很强；但传统GUI、原生Windows和部分任务性能不必然优于Gaussian/ORCA。</x:v>
       </x:c>
       <x:c r="E6" s="70" t="n">
-        <x:f>COUNTA('核心文献'!A5:A68)</x:f>
-        <x:v>64</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F6" s="70"/>
       <x:c r="G6" s="77" t="n">
-        <x:f>COUNTIF('核心文献'!B5:B68,"A")</x:f>
-        <x:v>25</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H6" s="77"/>
     </x:row>
@@ -1033,7 +991,7 @@
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="C9" s="33" t="str">
-        <x:v>先做科学完整性与跨代码验证，再做多引擎适配和高级场类型；问卷应询问过去12个月实际行为、选择因素、信任证据和采用障碍，而不是直接问“PySCF是否被认可”。</x:v>
+        <x:v>先完成多格式与科学完整性验证，再扩展多引擎适配和高级场类型；问卷优先测量过去12个月实际格式、首选格式、失败后果、元数据和采用门槛。</x:v>
       </x:c>
       <x:c r="E9" s="63" t="str">
         <x:v>软件矩阵</x:v>
@@ -1051,8 +1009,7 @@
       </x:c>
       <x:c r="F10" s="84"/>
       <x:c r="G10" s="84" t="n">
-        <x:f>COUNTA('问卷题库'!A5:A31)</x:f>
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="H10" s="84"/>
     </x:row>
@@ -1125,8 +1082,7 @@
         <x:v>互操作与工作流</x:v>
       </x:c>
       <x:c r="B20" s="30" t="n">
-        <x:f>COUNTIF('核心文献'!D5:D68,A20)</x:f>
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
@@ -1134,8 +1090,7 @@
         <x:v>数据格式与可视化</x:v>
       </x:c>
       <x:c r="B21" s="30" t="n">
-        <x:f>COUNTIF('核心文献'!D5:D68,A21)</x:f>
-        <x:v>12</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -1256,7 +1211,7 @@
     <x:mergeCell ref="A25:H25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3788292633a7457d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c90e40c50b9453d"/>
 </x:worksheet>
 </file>
 
@@ -4748,6 +4703,430 @@
         <x:v>便利样本、地区偏差、多选；谨慎引用。</x:v>
       </x:c>
     </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>L065</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>同行评议·可视化论文</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>数据格式与可视化</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>量子化学体数据</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>Interactive volume rendering of functional representations in quantum chemistry</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>Yun Jang; U. Varetto</x:v>
+      </x:c>
+      <x:c r="H69" t="n">
+        <x:v>2009</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>IEEE Transactions on Visualization and Computer Graphics</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>15(6), 1579–1586</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>10.1109/TVCG.2009.158</x:v>
+      </x:c>
+      <x:c r="L69" t="str">
+        <x:v>可视化方法论文</x:v>
+      </x:c>
+      <x:c r="M69" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>直接从基函数表示交互评估并体渲染量子化学场，讨论重采样与传输限制</x:v>
+      </x:c>
+      <x:c r="O69" t="str">
+        <x:v>问卷需同时测量文件型网格工作流与直接计算/交互工作流的需求。</x:v>
+      </x:c>
+      <x:c r="P69" t="str">
+        <x:v>https://doi.org/10.1109/TVCG.2009.158</x:v>
+      </x:c>
+      <x:c r="Q69" t="str">
+        <x:v>WoS定向筛选；待全文精读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>L066</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>同行评议·可视化论文</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>数据格式与可视化</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>量子化学体数据</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>Interactive visualization of quantum-chemistry data</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Yun Jang; Ugo Varetto</x:v>
+      </x:c>
+      <x:c r="H70" t="n">
+        <x:v>2010</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>Acta Crystallographica Section A</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>66(5), 542–552</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>10.1107/S010876731002636X</x:v>
+      </x:c>
+      <x:c r="L70" t="str">
+        <x:v>可视化方法论文</x:v>
+      </x:c>
+      <x:c r="M70" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N70" t="str">
+        <x:v>以GPU直接评估波函数并使用传递函数、裁剪和体渲染交互探索量子化学数据</x:v>
+      </x:c>
+      <x:c r="O70" t="str">
+        <x:v>产品概念不应局限于固定等值面；需询问交互阈值、裁剪和体渲染。</x:v>
+      </x:c>
+      <x:c r="P70" t="str">
+        <x:v>https://doi.org/10.1107/S010876731002636X</x:v>
+      </x:c>
+      <x:c r="Q70" t="str">
+        <x:v>WoS定向筛选；待全文精读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>L067</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>同行评议·综述</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>数据格式与可视化</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>交互量子化学</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>Interactive quantum chemistry enabled by machine learning, graphical processing units, and cloud computing</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>Umberto Raucci et al.</x:v>
+      </x:c>
+      <x:c r="H71" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>Annual Review of Physical Chemistry</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>74(1), 313–336</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>10.1146/annurev-physchem-061020-053438</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>综述</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>总结GPU、云端、机器学习输入和扩展现实如何降低实时计算与可视化门槛</x:v>
+      </x:c>
+      <x:c r="O71" t="str">
+        <x:v>问卷需区分科学能力与安装、编程、硬件、交互界面等采用障碍。</x:v>
+      </x:c>
+      <x:c r="P71" t="str">
+        <x:v>https://doi.org/10.1146/annurev-physchem-061020-053438</x:v>
+      </x:c>
+      <x:c r="Q71" t="str">
+        <x:v>WoS定向筛选；待全文精读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>L068</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>同行评议·应用论文</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>数据格式与可视化</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>增强现实</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>Bringing chemical structures to life with augmented reality, machine learning, and quantum chemistry</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>Sukolsak Sakshuwong et al.</x:v>
+      </x:c>
+      <x:c r="H72" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>Journal of Chemical Physics</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>156(20), 204801</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>10.1063/5.0090482</x:v>
+      </x:c>
+      <x:c r="L72" t="str">
+        <x:v>应用论文</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>展示低门槛移动端AR、名称/结构输入和云端量子化学属性计算</x:v>
+      </x:c>
+      <x:c r="O72" t="str">
+        <x:v>沉浸式呈现是交付形态之一，但不能替代可追溯的科学数据与验证。</x:v>
+      </x:c>
+      <x:c r="P72" t="str">
+        <x:v>https://doi.org/10.1063/5.0090482</x:v>
+      </x:c>
+      <x:c r="Q72" t="str">
+        <x:v>WoS定向筛选；摘要级证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>L069</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>同行评议·软件论文</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>数据格式与可视化</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>ORBKIT</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>ORBKIT: A modular Python toolbox for cross-platform postprocessing of quantum chemical wavefunction data</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>Gunter Hermann et al.</x:v>
+      </x:c>
+      <x:c r="H73" t="n">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>Journal of Computational Chemistry</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>37(16), 1511–1520</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>10.1002/jcc.24358</x:v>
+      </x:c>
+      <x:c r="L73" t="str">
+        <x:v>软件论文</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>从多种程序输出读取波函数，在任意网格计算密度、轨道与导数并输出多种可视化格式</x:v>
+      </x:c>
+      <x:c r="O73" t="str">
+        <x:v>格式需求应与源程序解耦，并覆盖波函数文件、规则网格和派生格式。</x:v>
+      </x:c>
+      <x:c r="P73" t="str">
+        <x:v>https://doi.org/10.1002/jcc.24358</x:v>
+      </x:c>
+      <x:c r="Q73" t="str">
+        <x:v>WoS定向筛选；待全文精读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>L070</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>同行评议·软件论文</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>互操作与工作流</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>QCDB/QCEngine</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>Quantum chemistry common driver and databases (QCDB) and Quantum Chemistry Engine (QCEngine): automation and interoperability among computational chemistry programs</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>Daniel G. A. Smith et al.</x:v>
+      </x:c>
+      <x:c r="H74" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>Journal of Chemical Physics</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>155(20), 204801</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>10.1063/5.0059356</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>软件/互操作论文</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>通过公共API统一多个量子化学程序的能量、梯度、Hessian和性质计算</x:v>
+      </x:c>
+      <x:c r="O74" t="str">
+        <x:v>问卷中的引擎无关概念应测量标准接口、统一变量和端到端自动化的价值。</x:v>
+      </x:c>
+      <x:c r="P74" t="str">
+        <x:v>https://doi.org/10.1063/5.0059356</x:v>
+      </x:c>
+      <x:c r="Q74" t="str">
+        <x:v>WoS定向筛选；待全文精读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>L071</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>同行评议·格式论文</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>互操作与工作流</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>QC-ML/HDF5</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>The problem of interoperability: A common data format for quantum chemistry codes</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>C. Angeli et al.</x:v>
+      </x:c>
+      <x:c r="H75" t="n">
+        <x:v>2007</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>International Journal of Quantum Chemistry</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>107(11), 2082–2091</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>10.1002/qua.21387</x:v>
+      </x:c>
+      <x:c r="L75" t="str">
+        <x:v>数据格式论文</x:v>
+      </x:c>
+      <x:c r="M75" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>以XML表达几何和基组等语义，以HDF5保存大型二进制数据</x:v>
+      </x:c>
+      <x:c r="O75" t="str">
+        <x:v>格式选择题必须把原始计算语义、波函数数据和派生体数据分开。</x:v>
+      </x:c>
+      <x:c r="P75" t="str">
+        <x:v>https://doi.org/10.1002/qua.21387</x:v>
+      </x:c>
+      <x:c r="Q75" t="str">
+        <x:v>WoS定向筛选；待全文精读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>L072</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>同行评议·软件论文</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>互操作与工作流</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>QMflows</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>QMflows: A tool kit for interoperable parallel workflows in quantum chemistry</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>Felipe Zapata et al.</x:v>
+      </x:c>
+      <x:c r="H76" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>Journal of Chemical Information and Modeling</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>59(7), 3191–3197</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>10.1021/acs.jcim.9b00384</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>工作流软件论文</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>以Python标准接口组织多个量子化学程序的并行工作流</x:v>
+      </x:c>
+      <x:c r="O76" t="str">
+        <x:v>交付方式需同时考虑脚本/API、HPC批处理和可扩展适配器。</x:v>
+      </x:c>
+      <x:c r="P76" t="str">
+        <x:v>https://doi.org/10.1021/acs.jcim.9b00384</x:v>
+      </x:c>
+      <x:c r="Q76" t="str">
+        <x:v>WoS定向筛选；摘要级证据。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
@@ -4771,7 +5150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf232e36050674e25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb74f4e55998f418b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5855,7 +6234,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56eb368a97364464"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc951d5d20f5b4cf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5890,7 +6269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>建议控制在8–10分钟；先问过去12个月实际行为，再问态度，避免直接引导“PySCF是否被认可”。</x:v>
+        <x:v>研究草案：预计12–15分钟。先问实际行为与文件格式，再问概念和PySCF次级变量；所有题目明确标注单选或多选。</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -5935,7 +6314,7 @@
         <x:v>Q01</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>筛选</x:v>
+        <x:v>背景</x:v>
       </x:c>
       <x:c r="C5" s="22" t="str">
         <x:v>您的主要工作身份是？</x:v>
@@ -5949,7 +6328,7 @@
       <x:c r="F5" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G5" s="22" t="str"/>
+      <x:c r="G5" s="22"/>
       <x:c r="H5" s="22" t="str">
         <x:v>样本分层</x:v>
       </x:c>
@@ -5962,7 +6341,7 @@
         <x:v>Q02</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>筛选</x:v>
+        <x:v>背景</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
         <x:v>您所在机构主要属于？</x:v>
@@ -5976,7 +6355,7 @@
       <x:c r="F6" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G6" s="22" t="str"/>
+      <x:c r="G6" s="22"/>
       <x:c r="H6" s="22" t="str">
         <x:v>行业分层</x:v>
       </x:c>
@@ -5998,12 +6377,12 @@
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E7" s="22" t="str">
-        <x:v>&lt;1；1–3；4–7；8–15；&gt;15年</x:v>
+        <x:v>不足1年；1–3年；4–7年；8–15年；超过15年</x:v>
       </x:c>
       <x:c r="F7" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G7" s="22" t="str"/>
+      <x:c r="G7" s="22"/>
       <x:c r="H7" s="22" t="str">
         <x:v>经验控制变量</x:v>
       </x:c>
@@ -6019,18 +6398,18 @@
         <x:v>背景</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
-        <x:v>您的主要研究对象是？</x:v>
+        <x:v>您的主要研究对象或工作场景有哪些？</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
-        <x:v>有机小分子；药物/生物分子；过渡金属/催化；激发态/光化学；固体/表面/二维材料；液体/界面；方法开发；教学；其他</x:v>
+        <x:v>有机小分子；药物/生物分子；过渡金属/催化；激发态/光化学；固体/表面/二维材料；液体/界面；方法开发；教学；科研软件开发；其他</x:v>
       </x:c>
       <x:c r="F8" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G8" s="22" t="str"/>
+      <x:c r="G8" s="22"/>
       <x:c r="H8" s="22" t="str">
         <x:v>领域分层</x:v>
       </x:c>
@@ -6043,10 +6422,10 @@
         <x:v>Q05</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>行为</x:v>
+        <x:v>实际工作流</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>过去12个月实际运行过哪些量子化学/电子结构程序？</x:v>
+        <x:v>过去12个月您实际运行过哪些量子化学/电子结构程序？</x:v>
       </x:c>
       <x:c r="D9" s="22" t="str">
         <x:v>多选</x:v>
@@ -6057,12 +6436,12 @@
       <x:c r="F9" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G9" s="22" t="str"/>
+      <x:c r="G9" s="22"/>
       <x:c r="H9" s="22" t="str">
-        <x:v>行为而非认知</x:v>
+        <x:v>实际使用</x:v>
       </x:c>
       <x:c r="I9" s="30" t="str">
-        <x:v>used_12m</x:v>
+        <x:v>used_engines_12m</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -6070,7 +6449,7 @@
         <x:v>Q06</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
-        <x:v>行为</x:v>
+        <x:v>实际工作流</x:v>
       </x:c>
       <x:c r="C10" s="22" t="str">
         <x:v>过去12个月您使用频率最高的主程序是？</x:v>
@@ -6079,12 +6458,12 @@
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>同Q05选项</x:v>
+        <x:v>沿用Q05选项；若Q05选择其他则显示其填写内容</x:v>
       </x:c>
       <x:c r="F10" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G10" s="22" t="str"/>
+      <x:c r="G10" s="22"/>
       <x:c r="H10" s="22" t="str">
         <x:v>主后端</x:v>
       </x:c>
@@ -6097,26 +6476,26 @@
         <x:v>Q07</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>行为</x:v>
+        <x:v>实际工作流</x:v>
       </x:c>
       <x:c r="C11" s="22" t="str">
-        <x:v>您通常如何使用主程序？</x:v>
+        <x:v>您通常通过哪些方式运行或组织计算？</x:v>
       </x:c>
       <x:c r="D11" s="22" t="str">
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E11" s="22" t="str">
-        <x:v>GUI；手写输入文件；Shell脚本；Python API/Notebook；工作流系统；云平台；他人代跑</x:v>
+        <x:v>GUI；手写输入文件；Shell/批处理脚本；Python API/Notebook；工作流系统；HPC调度系统；云平台；由他人代跑；其他</x:v>
       </x:c>
       <x:c r="F11" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G11" s="22" t="str"/>
+      <x:c r="G11" s="22"/>
       <x:c r="H11" s="22" t="str">
         <x:v>工作流模式</x:v>
       </x:c>
       <x:c r="I11" s="30" t="str">
-        <x:v>access_mode</x:v>
+        <x:v>access_modes</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -6124,26 +6503,26 @@
         <x:v>Q08</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>决策</x:v>
+        <x:v>实际工作流</x:v>
       </x:c>
       <x:c r="C12" s="22" t="str">
-        <x:v>选择计算程序时，请评价以下因素的重要性。</x:v>
+        <x:v>过去12个月您进行量子化学/电子结构计算的频率约为？</x:v>
       </x:c>
       <x:c r="D12" s="22" t="str">
-        <x:v>矩阵5点量表</x:v>
+        <x:v>单选</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
-        <x:v>数值可靠性；已有文献/同行采用；方法覆盖；速度；GPU/HPC；易安装；GUI；Python/API；许可成本；商业支持；开源可审计；与现有流程兼容</x:v>
+        <x:v>少于每月1次；每月1–3次；每周1–3次；每周4次以上；几乎每天；不确定</x:v>
       </x:c>
       <x:c r="F12" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G12" s="22" t="str"/>
+      <x:c r="G12" s="22"/>
       <x:c r="H12" s="22" t="str">
-        <x:v>选择驱动因素</x:v>
+        <x:v>使用强度</x:v>
       </x:c>
       <x:c r="I12" s="30" t="str">
-        <x:v>choice_factors</x:v>
+        <x:v>compute_frequency</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -6151,26 +6530,26 @@
         <x:v>Q09</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>信任</x:v>
+        <x:v>选择因素</x:v>
       </x:c>
       <x:c r="C13" s="22" t="str">
-        <x:v>什么证据最能提高您对一个量子化学程序结果的信任？</x:v>
+        <x:v>选择计算程序时，以下因素对您有多重要？</x:v>
       </x:c>
       <x:c r="D13" s="22" t="str">
-        <x:v>最多选3项</x:v>
+        <x:v>矩阵单选（每行5点）</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
-        <x:v>同行评议软件论文；独立跨代码基准；与实验吻合；源代码可见；自动测试；长期版本稳定；实验室/同事惯例；厂商支持；高引用量；大型用户群</x:v>
+        <x:v>行：数值可靠性；方法覆盖；速度；GPU/HPC；易安装；GUI；Python/API；许可成本；支持；开源可审计；现有流程兼容。列：完全不重要–非常重要；不了解</x:v>
       </x:c>
       <x:c r="F13" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G13" s="22" t="str"/>
+      <x:c r="G13" s="22"/>
       <x:c r="H13" s="22" t="str">
-        <x:v>认可度构成</x:v>
+        <x:v>选择驱动因素</x:v>
       </x:c>
       <x:c r="I13" s="30" t="str">
-        <x:v>trust_evidence</x:v>
+        <x:v>choice_factors</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -6178,26 +6557,26 @@
         <x:v>Q10</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>认知</x:v>
+        <x:v>可信度</x:v>
       </x:c>
       <x:c r="C14" s="22" t="str">
-        <x:v>在本问卷前，您对PySCF的了解程度？</x:v>
+        <x:v>哪些证据最能提高您对一个程序计算结果的信任？</x:v>
       </x:c>
       <x:c r="D14" s="22" t="str">
-        <x:v>单选</x:v>
+        <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
-        <x:v>未听说；听说但不了解；读过论文/文档；试用过；经常使用；参与开发</x:v>
+        <x:v>同行评议软件论文；独立跨程序基准；与实验吻合；公开源代码；自动测试；长期版本稳定；实验室/同事惯例；厂商支持；高引用量；大型用户群；其他</x:v>
       </x:c>
       <x:c r="F14" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G14" s="22" t="str"/>
+      <x:c r="G14" s="22"/>
       <x:c r="H14" s="22" t="str">
-        <x:v>PySCF漏斗</x:v>
+        <x:v>信任依据</x:v>
       </x:c>
       <x:c r="I14" s="30" t="str">
-        <x:v>pyscf_awareness</x:v>
+        <x:v>trust_evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -6205,28 +6584,26 @@
         <x:v>Q11</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>PySCF使用</x:v>
+        <x:v>可信度</x:v>
       </x:c>
       <x:c r="C15" s="22" t="str">
-        <x:v>您过去12个月是否实际运行过PySCF？</x:v>
+        <x:v>您会多频繁地用另一程序或独立流程交叉核验重要结果？</x:v>
       </x:c>
       <x:c r="D15" s="22" t="str">
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E15" s="22" t="str">
-        <x:v>是；否</x:v>
+        <x:v>从不；仅在异常时；仅在投稿/交付前；部分关键项目；多数项目；几乎每个项目</x:v>
       </x:c>
       <x:c r="F15" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G15" s="22" t="str">
-        <x:v>是→Q12；否→Q16</x:v>
-      </x:c>
+      <x:c r="G15" s="22"/>
       <x:c r="H15" s="22" t="str">
-        <x:v>使用分支</x:v>
+        <x:v>验证行为</x:v>
       </x:c>
       <x:c r="I15" s="30" t="str">
-        <x:v>pyscf_used</x:v>
+        <x:v>crosscheck_frequency</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
@@ -6234,28 +6611,28 @@
         <x:v>Q12</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>PySCF使用</x:v>
+        <x:v>可信度</x:v>
       </x:c>
       <x:c r="C16" s="22" t="str">
-        <x:v>您使用PySCF的任务有哪些？</x:v>
+        <x:v>过去12个月您使用哪些程序或方法做过交叉核验？</x:v>
       </x:c>
       <x:c r="D16" s="22" t="str">
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E16" s="22" t="str">
-        <x:v>HF/DFT；MP2/CC；CASSCF/多参考；激发态；周期体系；QM/MM；性质/谱学；方法开发；数据集/机器学习；教学；其他</x:v>
+        <x:v>Gaussian；ORCA；PySCF；Psi4；Q-Chem；Molpro/CFOUR；VASP/Quantum ESPRESSO/CP2K；自写实现；实验数据；公开基准集；其他；未做过</x:v>
       </x:c>
       <x:c r="F16" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="G16" s="22" t="str">
-        <x:v>仅Q11=是</x:v>
+        <x:v>Q11=从不者可直接选择“未做过”</x:v>
       </x:c>
       <x:c r="H16" s="22" t="str">
-        <x:v>实际场景</x:v>
+        <x:v>核验对象</x:v>
       </x:c>
       <x:c r="I16" s="30" t="str">
-        <x:v>pyscf_tasks</x:v>
+        <x:v>crosscheck_methods</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -6263,28 +6640,26 @@
         <x:v>Q13</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>PySCF评价</x:v>
+        <x:v>风险</x:v>
       </x:c>
       <x:c r="C17" s="22" t="str">
-        <x:v>请评价PySCF在以下方面的表现。</x:v>
+        <x:v>若可视化或格式转换出错，您实际担心哪些后果？</x:v>
       </x:c>
       <x:c r="D17" s="22" t="str">
-        <x:v>矩阵5点量表+不了解</x:v>
+        <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E17" s="22" t="str">
-        <x:v>数值可信；方法覆盖；性能；Python可编程性；文档；安装；报错可诊断性；版本稳定；GPU；与其他工具互操作</x:v>
+        <x:v>误判轨道/相位；误判密度或静电势；坐标/单位错误；周期边界错误；图像无法复现；批量任务静默失败；论文图或汇报返工；结论受影响；仅影响美观；其他</x:v>
       </x:c>
       <x:c r="F17" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G17" s="22" t="str">
-        <x:v>仅Q11=是</x:v>
-      </x:c>
+      <x:c r="G17" s="22"/>
       <x:c r="H17" s="22" t="str">
-        <x:v>优势/短板</x:v>
+        <x:v>失败后果</x:v>
       </x:c>
       <x:c r="I17" s="30" t="str">
-        <x:v>pyscf_rating</x:v>
+        <x:v>viz_failure_consequences</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
@@ -6292,28 +6667,26 @@
         <x:v>Q14</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>PySCF验证</x:v>
+        <x:v>可视化行为</x:v>
       </x:c>
       <x:c r="C18" s="22" t="str">
-        <x:v>您是否曾将PySCF结果与其他程序交叉验证？</x:v>
+        <x:v>过去12个月您使用过哪些工具查看轨道、密度或其他三维场？</x:v>
       </x:c>
       <x:c r="D18" s="22" t="str">
-        <x:v>单选+多选</x:v>
+        <x:v>多选</x:v>
       </x:c>
       <x:c r="E18" s="22" t="str">
-        <x:v>从未；Gaussian；ORCA；Psi4；Q-Chem；Molpro/CFOUR；其他</x:v>
+        <x:v>GaussView；Avogadro；VMD；PyMOL；Jmol/JSmol；Multiwfn；VESTA；OVITO；Blender插件；ParaView/VisIt；自写脚本；其他；未进行过此类可视化</x:v>
       </x:c>
       <x:c r="F18" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G18" s="22" t="str">
-        <x:v>仅Q11=是</x:v>
-      </x:c>
+      <x:c r="G18" s="22"/>
       <x:c r="H18" s="22" t="str">
-        <x:v>真实验证行为</x:v>
+        <x:v>现有方案</x:v>
       </x:c>
       <x:c r="I18" s="30" t="str">
-        <x:v>pyscf_crosscheck</x:v>
+        <x:v>viz_tools_12m</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
@@ -6321,28 +6694,26 @@
         <x:v>Q15</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>PySCF问题</x:v>
+        <x:v>可视化对象</x:v>
       </x:c>
       <x:c r="C19" s="22" t="str">
-        <x:v>您遇到过哪些PySCF障碍？</x:v>
+        <x:v>过去12个月您实际需要可视化哪些量？</x:v>
       </x:c>
       <x:c r="D19" s="22" t="str">
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E19" s="22" t="str">
-        <x:v>安装/Windows；收敛；默认设置不清；性能；缺少方法/性质；文档；GUI；输出后处理；团队不熟悉；许可/合规；无明显障碍；其他</x:v>
+        <x:v>分子轨道；总电子密度；自旋密度；静电势；差分密度；NTO/跃迁密度；ELF/LOL；局域轨道；周期电荷密度；能带/费米面；时间相关密度/波函数；拓扑临界点；其他；没有此需求</x:v>
       </x:c>
       <x:c r="F19" s="22" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="G19" s="22" t="str">
-        <x:v>仅Q11=是</x:v>
-      </x:c>
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G19" s="22"/>
       <x:c r="H19" s="22" t="str">
-        <x:v>采用障碍</x:v>
+        <x:v>场类型</x:v>
       </x:c>
       <x:c r="I19" s="30" t="str">
-        <x:v>pyscf_barriers_user</x:v>
+        <x:v>field_types</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -6350,28 +6721,26 @@
         <x:v>Q16</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>未使用原因</x:v>
+        <x:v>输入格式</x:v>
       </x:c>
       <x:c r="C20" s="22" t="str">
-        <x:v>您未使用PySCF的主要原因？</x:v>
+        <x:v>过去12个月您实际接收、生成或处理过哪些用于三维场/波函数可视化的文件格式？</x:v>
       </x:c>
       <x:c r="D20" s="22" t="str">
-        <x:v>最多选3项</x:v>
+        <x:v>多选</x:v>
       </x:c>
       <x:c r="E20" s="22" t="str">
-        <x:v>主程序已满足；不了解；缺少GUI；团队标准不是PySCF；担心认可度；担心数值一致性；安装/Windows；缺少所需方法；性能；商业支持；其他</x:v>
+        <x:v>Gaussian Cube（.cube/.cub）；Molden（.molden/.molden.input）；Gaussian formatted checkpoint（.fchk/.fch）；WFN/WFX（.wfn/.wfx）；XSF/AXSF/BXSF；OpenDX（.dx）；VASP体数据（CHGCAR/PARCHG/LOCPOT/ELFCAR）；CCP4/MRC密度图；VTK/VTI；自定义网格数组（CSV/NumPy/HDF5等）；OpenVDB（.vdb，派生可视化格式）；其他；未直接处理文件</x:v>
       </x:c>
       <x:c r="F20" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G20" s="22" t="str">
-        <x:v>仅Q11=否</x:v>
-      </x:c>
+      <x:c r="G20" s="22"/>
       <x:c r="H20" s="22" t="str">
-        <x:v>非用户障碍</x:v>
+        <x:v>实际格式覆盖</x:v>
       </x:c>
       <x:c r="I20" s="30" t="str">
-        <x:v>pyscf_barriers_nonuser</x:v>
+        <x:v>field_file_formats_12m</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
@@ -6379,26 +6748,26 @@
         <x:v>Q17</x:v>
       </x:c>
       <x:c r="B21" s="22" t="str">
-        <x:v>认可度</x:v>
+        <x:v>输入格式</x:v>
       </x:c>
       <x:c r="C21" s="22" t="str">
-        <x:v>在相同理论方法、基组/ECP、积分网格、收敛阈值和其他设置被严格统一且通过基准后，您是否愿意在论文/项目中采用PySCF结果？</x:v>
+        <x:v>如果只能优先支持一种输入格式，您最希望首先支持哪一种？</x:v>
       </x:c>
       <x:c r="D21" s="22" t="str">
-        <x:v>5点量表</x:v>
+        <x:v>单选</x:v>
       </x:c>
       <x:c r="E21" s="22" t="str">
-        <x:v>完全不愿意–完全愿意</x:v>
+        <x:v>沿用Q16选项，但不含“未直接处理文件”；另设“不确定/由工具自动识别即可”</x:v>
       </x:c>
       <x:c r="F21" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G21" s="22" t="str"/>
+      <x:c r="G21" s="22"/>
       <x:c r="H21" s="22" t="str">
-        <x:v>去除品牌混杂后的接受度</x:v>
+        <x:v>格式首要优先级</x:v>
       </x:c>
       <x:c r="I21" s="30" t="str">
-        <x:v>pyscf_accept_controlled</x:v>
+        <x:v>top_input_format</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
@@ -6406,26 +6775,26 @@
         <x:v>Q18</x:v>
       </x:c>
       <x:c r="B22" s="22" t="str">
-        <x:v>认可度</x:v>
+        <x:v>可视化行为</x:v>
       </x:c>
       <x:c r="C22" s="22" t="str">
-        <x:v>以下哪一项最接近您的看法？</x:v>
+        <x:v>过去12个月您制作三维场可视化的频率约为？</x:v>
       </x:c>
       <x:c r="D22" s="22" t="str">
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E22" s="22" t="str">
-        <x:v>程序品牌本身决定可信度；主要由方法和协议决定；两者同等重要；取决于具体任务；不确定</x:v>
+        <x:v>从未；少于每月1次；每月1–3次；每周1–3次；每周4次以上；几乎每天</x:v>
       </x:c>
       <x:c r="F22" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G22" s="22" t="str"/>
+      <x:c r="G22" s="22"/>
       <x:c r="H22" s="22" t="str">
-        <x:v>品牌与协议观念</x:v>
+        <x:v>需求强度</x:v>
       </x:c>
       <x:c r="I22" s="30" t="str">
-        <x:v>brand_vs_protocol</x:v>
+        <x:v>viz_frequency</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
@@ -6433,26 +6802,26 @@
         <x:v>Q19</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>可视化行为</x:v>
+        <x:v>痛点</x:v>
       </x:c>
       <x:c r="C23" s="22" t="str">
-        <x:v>您目前使用哪些工具查看轨道、密度或其他三维场？</x:v>
+        <x:v>当前三维场可视化中最耗时或最容易出错的环节有哪些？</x:v>
       </x:c>
       <x:c r="D23" s="22" t="str">
-        <x:v>多选</x:v>
+        <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E23" s="22" t="str">
-        <x:v>GaussView；Avogadro；VMD；PyMOL；Jmol/JSmol；Multiwfn/VMD；VESTA；Blender插件；自写脚本；其他；不使用</x:v>
+        <x:v>从计算结果提取/转换格式；单位/坐标/周期边界；选择等值面阈值；正负相位；多个态/轨道管理；批量处理；动画；材质/灯光；复现参数；超大网格内存；软件兼容；其他；无明显痛点</x:v>
       </x:c>
       <x:c r="F23" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G23" s="22" t="str"/>
+      <x:c r="G23" s="22"/>
       <x:c r="H23" s="22" t="str">
-        <x:v>竞品与工作流</x:v>
+        <x:v>核心痛点</x:v>
       </x:c>
       <x:c r="I23" s="30" t="str">
-        <x:v>viz_tools</x:v>
+        <x:v>viz_pain_points</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
@@ -6460,26 +6829,26 @@
         <x:v>Q20</x:v>
       </x:c>
       <x:c r="B24" s="22" t="str">
-        <x:v>可视化对象</x:v>
+        <x:v>元数据</x:v>
       </x:c>
       <x:c r="C24" s="22" t="str">
-        <x:v>您实际需要可视化哪些量？</x:v>
+        <x:v>为使一张三维场图可复核，您认为至少应随图保存哪些信息？</x:v>
       </x:c>
       <x:c r="D24" s="22" t="str">
-        <x:v>多选</x:v>
+        <x:v>多选（最多6项）</x:v>
       </x:c>
       <x:c r="E24" s="22" t="str">
-        <x:v>分子轨道；总电子密度；自旋密度；静电势；差分密度；NTO/跃迁密度；ELF/LOL；局域轨道；周期电荷密度；时间相关密度/波函数；拓扑临界点；其他</x:v>
+        <x:v>源程序及版本；方法/泛函；基组/ECP/赝势；电荷与自旋；网格原点和三个轴向量；单位；场类型及轨道/态索引；等值面/传递函数参数；原始文件哈希；转换工具版本；完整输入/输出链接；其他</x:v>
       </x:c>
       <x:c r="F24" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G24" s="22" t="str"/>
+      <x:c r="G24" s="22"/>
       <x:c r="H24" s="22" t="str">
-        <x:v>功能优先级</x:v>
+        <x:v>最低元数据</x:v>
       </x:c>
       <x:c r="I24" s="30" t="str">
-        <x:v>field_types</x:v>
+        <x:v>minimum_metadata</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
@@ -6487,26 +6856,26 @@
         <x:v>Q21</x:v>
       </x:c>
       <x:c r="B25" s="22" t="str">
-        <x:v>痛点</x:v>
+        <x:v>概念测试</x:v>
       </x:c>
       <x:c r="C25" s="22" t="str">
-        <x:v>当前量子化学可视化中最耗时或最容易出错的环节是什么？</x:v>
+        <x:v>设想一个与具体计算程序无关的工具：它读取多种量子化学场/波函数文件，保留计算元数据，检查单位、坐标和网格，并生成可复现的Blender/OpenVDB场景。您认为它对自己的工作有多大价值？</x:v>
       </x:c>
       <x:c r="D25" s="22" t="str">
-        <x:v>最多选3项</x:v>
+        <x:v>单选（5点量表）</x:v>
       </x:c>
       <x:c r="E25" s="22" t="str">
-        <x:v>计算到格式转换；单位/坐标/周期边界；选择等值面阈值；正负相位；批量处理；动画；材质/灯光；复现实验参数；超大网格内存；软件兼容；其他</x:v>
+        <x:v>完全无价值；价值较低；一般；价值较高；非常有价值；信息不足无法判断</x:v>
       </x:c>
       <x:c r="F25" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G25" s="22" t="str"/>
+      <x:c r="G25" s="22"/>
       <x:c r="H25" s="22" t="str">
-        <x:v>产品问题验证</x:v>
+        <x:v>概念价值</x:v>
       </x:c>
       <x:c r="I25" s="30" t="str">
-        <x:v>viz_pain</x:v>
+        <x:v>pipeline_value</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
@@ -6514,26 +6883,26 @@
         <x:v>Q22</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>概念测试</x:v>
+        <x:v>功能优先级</x:v>
       </x:c>
       <x:c r="C26" s="22" t="str">
-        <x:v>一个“引擎无关”的工具可从PySCF/Gaussian/ORCA等读取计算与元数据，验证cube/场数据，生成OpenVDB并在Blender中自动创建可复现场景。您认为其价值如何？</x:v>
+        <x:v>请选出您最需要的5项功能。</x:v>
       </x:c>
       <x:c r="D26" s="22" t="str">
-        <x:v>5点量表</x:v>
+        <x:v>多选（最多5项）</x:v>
       </x:c>
       <x:c r="E26" s="22" t="str">
-        <x:v>完全无价值–非常有价值</x:v>
+        <x:v>多格式输入；保留完整计算元数据；数值校验报告；一键Blender场景；交互等值面/体渲染；正负轨道叶分离；周期单胞/超胞；多帧动画；NTO/差分密度；大网格稀疏VDB；批处理；Python API；GUI；自动图注；原始文件哈希归档</x:v>
       </x:c>
       <x:c r="F26" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G26" s="22" t="str"/>
+      <x:c r="G26" s="22"/>
       <x:c r="H26" s="22" t="str">
-        <x:v>价值主张</x:v>
+        <x:v>路线图</x:v>
       </x:c>
       <x:c r="I26" s="30" t="str">
-        <x:v>pipeline_value</x:v>
+        <x:v>feature_priority</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -6541,26 +6910,26 @@
         <x:v>Q23</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>功能排序</x:v>
+        <x:v>验证门槛</x:v>
       </x:c>
       <x:c r="C27" s="22" t="str">
-        <x:v>请选出最重要的5项功能。</x:v>
+        <x:v>对于从原始场文件到派生可视化格式的转换，哪些验证是您采用该工具的最低要求？</x:v>
       </x:c>
       <x:c r="D27" s="22" t="str">
-        <x:v>最多选5项</x:v>
+        <x:v>多选</x:v>
       </x:c>
       <x:c r="E27" s="22" t="str">
-        <x:v>保留完整计算元数据；数值校验报告；多程序输入；一键Blender场景；正负轨道叶分离；周期单胞/超胞；多帧动画；NTO/差分密度；大网格稀疏VDB；批处理；Python API；GUI；自动生成方法说明/图注；原始文件哈希归档</x:v>
+        <x:v>坐标/仿射变换一致；最大/RMS场误差；积分量或电子数；正负符号保持；周期端点检查；等值面面积/体积对照；原始文件哈希；软件/版本/方法元数据；自动回归测试；人工视觉检查即可；其他</x:v>
       </x:c>
       <x:c r="F27" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G27" s="22" t="str"/>
+      <x:c r="G27" s="22"/>
       <x:c r="H27" s="22" t="str">
-        <x:v>路线图排序</x:v>
+        <x:v>验收要求</x:v>
       </x:c>
       <x:c r="I27" s="30" t="str">
-        <x:v>feature_priority</x:v>
+        <x:v>validation_minimum</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
@@ -6568,26 +6937,26 @@
         <x:v>Q24</x:v>
       </x:c>
       <x:c r="B28" s="22" t="str">
-        <x:v>验证门槛</x:v>
+        <x:v>交付方式</x:v>
       </x:c>
       <x:c r="C28" s="22" t="str">
-        <x:v>您接受cube→VDB转换的最低验证要求？</x:v>
+        <x:v>您可能采用哪些交付方式？</x:v>
       </x:c>
       <x:c r="D28" s="22" t="str">
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E28" s="22" t="str">
-        <x:v>坐标/仿射变换一致；最大/RMS场误差；积分电子数；正负符号保持；等值面面积/体积对照；原始cube哈希；软件/版本/方法元数据；视觉检查即可；其他</x:v>
+        <x:v>Blender插件；独立CLI；Python包；Jupyter界面；桌面GUI；Web服务；HPC批处理；容器镜像；机构内部部署；其他</x:v>
       </x:c>
       <x:c r="F28" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G28" s="22" t="str"/>
+      <x:c r="G28" s="22"/>
       <x:c r="H28" s="22" t="str">
-        <x:v>验收标准</x:v>
+        <x:v>产品形态</x:v>
       </x:c>
       <x:c r="I28" s="30" t="str">
-        <x:v>validation_minimum</x:v>
+        <x:v>delivery_modes</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
@@ -6595,26 +6964,26 @@
         <x:v>Q25</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>部署</x:v>
+        <x:v>采用门槛</x:v>
       </x:c>
       <x:c r="C29" s="22" t="str">
-        <x:v>您更可能采用哪种交付方式？</x:v>
+        <x:v>以下哪项最可能成为您不采用该工具的首要原因？</x:v>
       </x:c>
       <x:c r="D29" s="22" t="str">
-        <x:v>多选</x:v>
+        <x:v>单选</x:v>
       </x:c>
       <x:c r="E29" s="22" t="str">
-        <x:v>Blender插件；独立CLI；Python包；Jupyter界面；Web服务；HPC批处理；容器镜像；机构内部部署</x:v>
+        <x:v>不支持现有文件格式；难以安装；缺少GUI；无法在HPC/离线环境运行；缺少科学验证；处理大文件太慢；不能批量自动化；许可证/合规问题；团队已有稳定方案；没有足够需求；其他</x:v>
       </x:c>
       <x:c r="F29" s="22" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="G29" s="22" t="str"/>
+      <x:c r="G29" s="22"/>
       <x:c r="H29" s="22" t="str">
-        <x:v>产品形态</x:v>
+        <x:v>首要采用障碍</x:v>
       </x:c>
       <x:c r="I29" s="30" t="str">
-        <x:v>delivery</x:v>
+        <x:v>top_adoption_barrier</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
@@ -6622,24 +6991,26 @@
         <x:v>Q26</x:v>
       </x:c>
       <x:c r="B30" s="22" t="str">
-        <x:v>开放</x:v>
+        <x:v>PySCF次级变量</x:v>
       </x:c>
       <x:c r="C30" s="22" t="str">
-        <x:v>请描述一个当前工具难以完成、但您希望该工作流解决的具体案例。</x:v>
+        <x:v>在本问卷前，您对PySCF的了解程度？</x:v>
       </x:c>
       <x:c r="D30" s="22" t="str">
-        <x:v>开放题</x:v>
-      </x:c>
-      <x:c r="E30" s="22" t="str"/>
+        <x:v>单选</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="str">
+        <x:v>未听说；听说但不了解；读过论文/文档；试用过；经常使用；参与开发</x:v>
+      </x:c>
       <x:c r="F30" s="22" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="G30" s="22" t="str"/>
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G30" s="22"/>
       <x:c r="H30" s="22" t="str">
-        <x:v>需求发现</x:v>
+        <x:v>认知漏斗</x:v>
       </x:c>
       <x:c r="I30" s="30" t="str">
-        <x:v>open_case</x:v>
+        <x:v>pyscf_awareness</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
@@ -6647,26 +7018,113 @@
         <x:v>Q27</x:v>
       </x:c>
       <x:c r="B31" s="32" t="str">
-        <x:v>招募</x:v>
+        <x:v>PySCF次级变量</x:v>
       </x:c>
       <x:c r="C31" s="32" t="str">
-        <x:v>您是否愿意参加后续30分钟访谈或提供匿名测试数据？</x:v>
+        <x:v>过去12个月您是否实际运行过PySCF？</x:v>
       </x:c>
       <x:c r="D31" s="32" t="str">
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
-        <x:v>愿意访谈；愿意提供测试数据；两者都愿意；暂不愿意</x:v>
+        <x:v>是；否</x:v>
       </x:c>
       <x:c r="F31" s="32" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G31" s="32" t="str">
+        <x:v>是→Q28；否→Q29</x:v>
+      </x:c>
+      <x:c r="H31" s="32" t="str">
+        <x:v>实际使用</x:v>
+      </x:c>
+      <x:c r="I31" s="33" t="str">
+        <x:v>pyscf_used_12m</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="61.5" customHeight="1">
+      <x:c r="A32" s="108" t="str">
+        <x:v>Q28</x:v>
+      </x:c>
+      <x:c r="B32" s="108" t="str">
+        <x:v>PySCF次级变量</x:v>
+      </x:c>
+      <x:c r="C32" s="108" t="str">
+        <x:v>您在使用PySCF时遇到过哪些障碍？</x:v>
+      </x:c>
+      <x:c r="D32" s="108" t="str">
+        <x:v>多选</x:v>
+      </x:c>
+      <x:c r="E32" s="108" t="str">
+        <x:v>安装/Windows；收敛；默认设置不清；性能；缺少方法/性质；文档；GUI；输出后处理；团队不熟悉；许可/合规；无明显障碍；其他</x:v>
+      </x:c>
+      <x:c r="F32" s="108" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G32" s="108" t="str">
+        <x:v>仅Q27=是；完成后→Q30</x:v>
+      </x:c>
+      <x:c r="H32" s="108" t="str">
+        <x:v>用户障碍</x:v>
+      </x:c>
+      <x:c r="I32" s="108" t="str">
+        <x:v>pyscf_user_barriers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="61.5" customHeight="1">
+      <x:c r="A33" s="108" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B33" s="108" t="str">
+        <x:v>PySCF次级变量</x:v>
+      </x:c>
+      <x:c r="C33" s="108" t="str">
+        <x:v>您未使用PySCF的主要原因有哪些？</x:v>
+      </x:c>
+      <x:c r="D33" s="108" t="str">
+        <x:v>多选（最多3项）</x:v>
+      </x:c>
+      <x:c r="E33" s="108" t="str">
+        <x:v>不了解；主程序已满足；缺少GUI；团队标准不是PySCF；担心认可度；担心数值一致性；安装/Windows；缺少所需方法；性能；商业支持；其他</x:v>
+      </x:c>
+      <x:c r="F33" s="108" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G33" s="108" t="str">
+        <x:v>仅Q27=否；完成后→Q30</x:v>
+      </x:c>
+      <x:c r="H33" s="108" t="str">
+        <x:v>非用户障碍</x:v>
+      </x:c>
+      <x:c r="I33" s="108" t="str">
+        <x:v>pyscf_nonuser_barriers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="39" customHeight="1">
+      <x:c r="A34" s="108" t="str">
+        <x:v>Q30</x:v>
+      </x:c>
+      <x:c r="B34" s="108" t="str">
+        <x:v>开放反馈</x:v>
+      </x:c>
+      <x:c r="C34" s="108" t="str">
+        <x:v>请描述一个当前工具难以完成、但您希望引擎无关可视化工作流解决的具体案例。</x:v>
+      </x:c>
+      <x:c r="D34" s="108" t="str">
+        <x:v>开放题</x:v>
+      </x:c>
+      <x:c r="E34" s="108" t="str">
+        <x:v>自由文本</x:v>
+      </x:c>
+      <x:c r="F34" s="108" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="G31" s="32" t="str"/>
-      <x:c r="H31" s="32" t="str">
-        <x:v>后续研究</x:v>
-      </x:c>
-      <x:c r="I31" s="33" t="str">
-        <x:v>followup</x:v>
+      <x:c r="G34" s="108"/>
+      <x:c r="H34" s="108" t="str">
+        <x:v>需求发现</x:v>
+      </x:c>
+      <x:c r="I34" s="108" t="str">
+        <x:v>open_case</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6681,7 +7139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77385f9da8c14a04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde91ece6f53245ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7422,7 +7880,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76bce2ce49094e4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde728ea175af44de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize literature-backed survey
</commit_message>
<xml_diff>
--- a/pyscf_quantum_chemistry_visualization_research_2026-07-19.xlsx
+++ b/pyscf_quantum_chemistry_visualization_research_2026-07-19.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R0b9e11b89d1f4ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心文献" sheetId="2" r:id="Rbe4ae855ed8f443f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件矩阵" sheetId="3" r:id="R47bbef6c080c43a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷题库" sheetId="4" r:id="R655fbeae2d1746fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验证矩阵" sheetId="5" r:id="Rd42fa0551dfb4bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rd20d26b660f34ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心文献" sheetId="2" r:id="Rc26356d27f45482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件矩阵" sheetId="3" r:id="R09beb7550d8444a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问卷题库" sheetId="4" r:id="Rf88f37b138614d25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验证矩阵" sheetId="5" r:id="R89da4d2e75a842d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -626,7 +626,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5fcfb790519d47e3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd5f7c5d4c04b49c3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -991,7 +991,7 @@
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="C9" s="33" t="str">
-        <x:v>先完成多格式与科学完整性验证，再扩展多引擎适配和高级场类型；问卷优先测量过去12个月实际格式、首选格式、失败后果、元数据和采用门槛。</x:v>
+        <x:v>关键全文已核验，问卷进入10–15人认知预测试；产品路线先完成多格式与科学完整性验证，再扩展多引擎适配和高级场类型。</x:v>
       </x:c>
       <x:c r="E9" s="63" t="str">
         <x:v>软件矩阵</x:v>
@@ -1211,7 +1211,7 @@
     <x:mergeCell ref="A25:H25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c90e40c50b9453d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eb9d65a9f584435"/>
 </x:worksheet>
 </file>
 
@@ -4741,19 +4741,19 @@
         <x:v>可视化方法论文</x:v>
       </x:c>
       <x:c r="M69" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N69" t="str">
-        <x:v>直接从基函数表示交互评估并体渲染量子化学场，讨论重采样与传输限制</x:v>
+        <x:v>直接从基函数表示交互评估并体渲染量子化学场，讨论规则网格重采样的存储、传输和分辨率限制</x:v>
       </x:c>
       <x:c r="O69" t="str">
-        <x:v>问卷需同时测量文件型网格工作流与直接计算/交互工作流的需求。</x:v>
+        <x:v>问卷需同时测量文件型网格工作流、直接场评估、传递函数、裁剪与体渲染需求。</x:v>
       </x:c>
       <x:c r="P69" t="str">
         <x:v>https://doi.org/10.1109/TVCG.2009.158</x:v>
       </x:c>
       <x:c r="Q69" t="str">
-        <x:v>WoS定向筛选；待全文精读。</x:v>
+        <x:v>WoS定向筛选；全文精读。与L066属于同一证据家族，综合时避免重复计权。</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -4794,10 +4794,10 @@
         <x:v>可视化方法论文</x:v>
       </x:c>
       <x:c r="M70" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N70" t="str">
-        <x:v>以GPU直接评估波函数并使用传递函数、裁剪和体渲染交互探索量子化学数据</x:v>
+        <x:v>以GPU直接评估波函数并使用切片、二维传递函数、裁剪和体渲染交互探索量子化学数据</x:v>
       </x:c>
       <x:c r="O70" t="str">
         <x:v>产品概念不应局限于固定等值面；需询问交互阈值、裁剪和体渲染。</x:v>
@@ -4806,7 +4806,7 @@
         <x:v>https://doi.org/10.1107/S010876731002636X</x:v>
       </x:c>
       <x:c r="Q70" t="str">
-        <x:v>WoS定向筛选；待全文精读。</x:v>
+        <x:v>WoS定向筛选；全文精读。与L065属于同一证据家族，综合时避免重复计权。</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -4847,10 +4847,10 @@
         <x:v>综述</x:v>
       </x:c>
       <x:c r="M71" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N71" t="str">
-        <x:v>总结GPU、云端、机器学习输入和扩展现实如何降低实时计算与可视化门槛</x:v>
+        <x:v>指出领域知识、编程、输入输出处理和高性能硬件是进入门槛，并总结GPU、云端、自然界面和扩展现实方案</x:v>
       </x:c>
       <x:c r="O71" t="str">
         <x:v>问卷需区分科学能力与安装、编程、硬件、交互界面等采用障碍。</x:v>
@@ -4859,7 +4859,7 @@
         <x:v>https://doi.org/10.1146/annurev-physchem-061020-053438</x:v>
       </x:c>
       <x:c r="Q71" t="str">
-        <x:v>WoS定向筛选；待全文精读。</x:v>
+        <x:v>WoS定向筛选；全文精读。</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -4900,7 +4900,7 @@
         <x:v>应用论文</x:v>
       </x:c>
       <x:c r="M72" t="str">
-        <x:v>待核对</x:v>
+        <x:v>摘要已核验</x:v>
       </x:c>
       <x:c r="N72" t="str">
         <x:v>展示低门槛移动端AR、名称/结构输入和云端量子化学属性计算</x:v>
@@ -4912,7 +4912,7 @@
         <x:v>https://doi.org/10.1063/5.0090482</x:v>
       </x:c>
       <x:c r="Q72" t="str">
-        <x:v>WoS定向筛选；摘要级证据。</x:v>
+        <x:v>WoS定向筛选；补充案例，不承担核心构念。</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -4953,19 +4953,19 @@
         <x:v>软件论文</x:v>
       </x:c>
       <x:c r="M73" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N73" t="str">
-        <x:v>从多种程序输出读取波函数，在任意网格计算密度、轨道与导数并输出多种可视化格式</x:v>
+        <x:v>从多种程序输出读取波函数，在任意网格计算密度、轨道与导数，并提供多种后处理输出</x:v>
       </x:c>
       <x:c r="O73" t="str">
-        <x:v>格式需求应与源程序解耦，并覆盖波函数文件、规则网格和派生格式。</x:v>
+        <x:v>格式需求应与源程序解耦，并覆盖波函数源格式、规则网格、任意网格控制和多帧轨道一致性。</x:v>
       </x:c>
       <x:c r="P73" t="str">
         <x:v>https://doi.org/10.1002/jcc.24358</x:v>
       </x:c>
       <x:c r="Q73" t="str">
-        <x:v>WoS定向筛选；待全文精读。</x:v>
+        <x:v>WoS定向筛选；全文精读。</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -5006,19 +5006,19 @@
         <x:v>软件/互操作论文</x:v>
       </x:c>
       <x:c r="M74" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N74" t="str">
-        <x:v>通过公共API统一多个量子化学程序的能量、梯度、Hessian和性质计算</x:v>
+        <x:v>用QCSchema JSON、验证、单位转换和程序适配器统一多程序输入输出，同时允许程序特定关键字</x:v>
       </x:c>
       <x:c r="O74" t="str">
-        <x:v>问卷中的引擎无关概念应测量标准接口、统一变量和端到端自动化的价值。</x:v>
+        <x:v>引擎无关概念应测量标准接口、统一变量、来源记录和保留程序特定控制的价值。</x:v>
       </x:c>
       <x:c r="P74" t="str">
         <x:v>https://doi.org/10.1063/5.0059356</x:v>
       </x:c>
       <x:c r="Q74" t="str">
-        <x:v>WoS定向筛选；待全文精读。</x:v>
+        <x:v>WoS定向筛选；替换附件已确认可提取全文并完成精读。</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -5059,10 +5059,10 @@
         <x:v>数据格式论文</x:v>
       </x:c>
       <x:c r="M75" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N75" t="str">
-        <x:v>以XML表达几何和基组等语义，以HDF5保存大型二进制数据</x:v>
+        <x:v>以XML表达几何、原子、基组、电荷、自旋和多状态等语义，以HDF5保存大型二进制数组并用schema验证</x:v>
       </x:c>
       <x:c r="O75" t="str">
         <x:v>格式选择题必须把原始计算语义、波函数数据和派生体数据分开。</x:v>
@@ -5071,7 +5071,7 @@
         <x:v>https://doi.org/10.1002/qua.21387</x:v>
       </x:c>
       <x:c r="Q75" t="str">
-        <x:v>WoS定向筛选；待全文精读。</x:v>
+        <x:v>WoS定向筛选；全文精读。</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -5112,19 +5112,19 @@
         <x:v>工作流软件论文</x:v>
       </x:c>
       <x:c r="M76" t="str">
-        <x:v>待核对</x:v>
+        <x:v>全文已核验</x:v>
       </x:c>
       <x:c r="N76" t="str">
-        <x:v>以Python标准接口组织多个量子化学程序的并行工作流</x:v>
+        <x:v>以Python标准接口组织输入准备、队列提交、结果收集和多程序并行工作流</x:v>
       </x:c>
       <x:c r="O76" t="str">
-        <x:v>交付方式需同时考虑脚本/API、HPC批处理和可扩展适配器。</x:v>
+        <x:v>交付方式需同时考虑脚本/API、HPC批处理、依赖管理和可扩展适配器。</x:v>
       </x:c>
       <x:c r="P76" t="str">
         <x:v>https://doi.org/10.1021/acs.jcim.9b00384</x:v>
       </x:c>
       <x:c r="Q76" t="str">
-        <x:v>WoS定向筛选；摘要级证据。</x:v>
+        <x:v>WoS定向筛选；全文精读。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5150,7 +5150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb74f4e55998f418b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38ca4bcf04d74bb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6234,7 +6234,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc951d5d20f5b4cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d93ea5943694a0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6269,7 +6269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>研究草案：预计12–15分钟。先问实际行为与文件格式，再问概念和PySCF次级变量；所有题目明确标注单选或多选。</x:v>
+        <x:v>文献支撑预测试版：预计12–15分钟。先问实际行为与文件格式，再问概念和PySCF次级变量；所有题目明确标注单选或多选。</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -6724,7 +6724,7 @@
         <x:v>输入格式</x:v>
       </x:c>
       <x:c r="C20" s="22" t="str">
-        <x:v>过去12个月您实际接收、生成或处理过哪些用于三维场/波函数可视化的文件格式？</x:v>
+        <x:v>过去12个月您实际接收、生成或处理过哪些用于三维场/波函数可视化的文件格式？下列同时包含波函数/轨道源格式、已采样体网格和派生可视化格式。</x:v>
       </x:c>
       <x:c r="D20" s="22" t="str">
         <x:v>多选</x:v>
@@ -6751,7 +6751,7 @@
         <x:v>输入格式</x:v>
       </x:c>
       <x:c r="C21" s="22" t="str">
-        <x:v>如果只能优先支持一种输入格式，您最希望首先支持哪一种？</x:v>
+        <x:v>如果工具首版只能优先适配一种输入或交换格式，您最希望首先支持哪一种？</x:v>
       </x:c>
       <x:c r="D21" s="22" t="str">
         <x:v>单选</x:v>
@@ -6811,7 +6811,7 @@
         <x:v>多选（最多3项）</x:v>
       </x:c>
       <x:c r="E23" s="22" t="str">
-        <x:v>从计算结果提取/转换格式；单位/坐标/周期边界；选择等值面阈值；正负相位；多个态/轨道管理；批量处理；动画；材质/灯光；复现参数；超大网格内存；软件兼容；其他；无明显痛点</x:v>
+        <x:v>从计算结果提取/转换格式；单位/坐标/周期边界；选择等值面阈值；交互传递函数/裁剪；正负相位；多个态/轨道及跨帧一致性；批量处理；动画；材质/灯光；复现参数；超大网格内存；软件兼容；其他；无明显痛点</x:v>
       </x:c>
       <x:c r="F23" s="22" t="str">
         <x:v>是</x:v>
@@ -6838,7 +6838,7 @@
         <x:v>多选（最多6项）</x:v>
       </x:c>
       <x:c r="E24" s="22" t="str">
-        <x:v>源程序及版本；方法/泛函；基组/ECP/赝势；电荷与自旋；网格原点和三个轴向量；单位；场类型及轨道/态索引；等值面/传递函数参数；原始文件哈希；转换工具版本；完整输入/输出链接；其他</x:v>
+        <x:v>源程序及版本；方法/泛函；基组/ECP/赝势；程序特定关键字及非默认设置；电荷与自旋；网格原点和三个轴向量；单位；场类型及轨道/态索引；等值面/传递函数参数；原始文件哈希；转换工具版本；完整输入/输出或计算记录链接；其他</x:v>
       </x:c>
       <x:c r="F24" s="22" t="str">
         <x:v>是</x:v>
@@ -6892,7 +6892,7 @@
         <x:v>多选（最多5项）</x:v>
       </x:c>
       <x:c r="E26" s="22" t="str">
-        <x:v>多格式输入；保留完整计算元数据；数值校验报告；一键Blender场景；交互等值面/体渲染；正负轨道叶分离；周期单胞/超胞；多帧动画；NTO/差分密度；大网格稀疏VDB；批处理；Python API；GUI；自动图注；原始文件哈希归档</x:v>
+        <x:v>多格式输入；保留完整计算元数据；保留程序特定控制并报告适配器能力；数值校验报告；一键Blender场景；交互等值面/体渲染/裁剪；正负轨道叶分离；周期单胞/超胞；多帧动画；NTO/差分密度；大网格稀疏VDB；批处理；Python API；GUI；自动图注；原始文件哈希归档</x:v>
       </x:c>
       <x:c r="F26" s="22" t="str">
         <x:v>是</x:v>
@@ -6919,7 +6919,7 @@
         <x:v>多选</x:v>
       </x:c>
       <x:c r="E27" s="22" t="str">
-        <x:v>坐标/仿射变换一致；最大/RMS场误差；积分量或电子数；正负符号保持；周期端点检查；等值面面积/体积对照；原始文件哈希；软件/版本/方法元数据；自动回归测试；人工视觉检查即可；其他</x:v>
+        <x:v>坐标/仿射变换一致；单位、数组形状与数据顺序检查；最大/RMS场误差；积分量或电子数；正负符号保持；周期端点检查；等值面面积/体积对照；原始文件哈希；软件/版本/方法/网格元数据；自动回归测试；人工视觉检查即可；其他</x:v>
       </x:c>
       <x:c r="F27" s="22" t="str">
         <x:v>是</x:v>
@@ -6973,7 +6973,7 @@
         <x:v>单选</x:v>
       </x:c>
       <x:c r="E29" s="22" t="str">
-        <x:v>不支持现有文件格式；难以安装；缺少GUI；无法在HPC/离线环境运行；缺少科学验证；处理大文件太慢；不能批量自动化；许可证/合规问题；团队已有稳定方案；没有足够需求；其他</x:v>
+        <x:v>不支持现有文件格式；难以安装；需要额外编程/脚本经验；缺少GUI；无法在HPC/离线环境运行；缺少科学验证；处理大文件太慢；不能批量自动化；许可证/合规问题；团队已有稳定方案；没有足够需求；其他</x:v>
       </x:c>
       <x:c r="F29" s="22" t="str">
         <x:v>是</x:v>
@@ -7139,7 +7139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde91ece6f53245ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4f1b89327e4369"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7880,7 +7880,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde728ea175af44de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red6389d6ee454492"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>